<commit_message>
modify lab-002 and add lab-003, lab-004
</commit_message>
<xml_diff>
--- a/jnciesproadmap/JNCIE-SP_Juniper_SP_Engineer_Lab_Roadmap.xlsx
+++ b/jnciesproadmap/JNCIE-SP_Juniper_SP_Engineer_Lab_Roadmap.xlsx
@@ -201,16 +201,16 @@
     <t xml:space="preserve">Filter, match, count, display detail/extensive, monitor, request support information and save evidence efficiently.</t>
   </si>
   <si>
+    <t>LAB-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Routing tables and next-hop resolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trace a route across inet.0, inet.3, mpls.0 and protocol-specific tables including hidden routes.</t>
+  </si>
+  <si>
     <t xml:space="preserve">☐ Not Started</t>
-  </si>
-  <si>
-    <t>LAB-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Routing tables and next-hop resolution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trace a route across inet.0, inet.3, mpls.0 and protocol-specific tables including hidden routes.</t>
   </si>
   <si>
     <t>LAB-005</t>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B6" s="8">
         <f>COUNTIF('Lab Checklist'!$L$2:$L$124,"*Completed*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="7">
@@ -2700,11 +2700,11 @@
       <c r="F6" s="9"/>
       <c r="G6" s="10">
         <f>IFERROR(B6/A6,0)</f>
-        <v>0.016260162601626018</v>
+        <v>0.024390243902439025</v>
       </c>
       <c r="H6" s="8">
         <f>SUMIF('Lab Checklist'!$L$2:$L$124,"*Completed*",'Lab Checklist'!$H$2:$H$124)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" ht="15">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="C9" s="16">
         <f>COUNTIFS('Lab Checklist'!$B$2:$B$124,A9,'Lab Checklist'!$L$2:$L$124,"*Completed*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="17">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.20000000000000001</v>
+        <v>0.29999999999999999</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>13</v>
@@ -2956,7 +2956,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" priority="2" id="{2F82F829-2141-4B30-A417-98EBA9B532D7}">
+          <x14:cfRule type="dataBar" priority="2" id="{F3328177-44D9-473A-BA9E-58720EA418BB}">
             <x14:dataBar maxLength="90" minLength="10" axisPosition="automatic" direction="context">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -3181,7 +3181,7 @@
         <v>51</v>
       </c>
       <c r="L4" s="23" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="M4" s="23">
         <v>0</v>
@@ -3195,7 +3195,7 @@
     </row>
     <row r="5" ht="38.25">
       <c r="A5" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>12</v>
@@ -3207,10 +3207,10 @@
         <v>43</v>
       </c>
       <c r="E5" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>59</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>60</v>
       </c>
       <c r="G5" s="24" t="s">
         <v>46</v>
@@ -3228,7 +3228,7 @@
         <v>54</v>
       </c>
       <c r="L5" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M5" s="23">
         <v>0</v>
@@ -3272,10 +3272,10 @@
         <v>48</v>
       </c>
       <c r="K6" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L6" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M6" s="23">
         <v>0</v>
@@ -3322,7 +3322,7 @@
         <v>61</v>
       </c>
       <c r="L7" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M7" s="23">
         <v>0</v>
@@ -3369,7 +3369,7 @@
         <v>64</v>
       </c>
       <c r="L8" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M8" s="23">
         <v>0</v>
@@ -3416,7 +3416,7 @@
         <v>67</v>
       </c>
       <c r="L9" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M9" s="23">
         <v>0</v>
@@ -3463,7 +3463,7 @@
         <v>70</v>
       </c>
       <c r="L10" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M10" s="23">
         <v>0</v>
@@ -3510,7 +3510,7 @@
         <v>73</v>
       </c>
       <c r="L11" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M11" s="23">
         <v>0</v>
@@ -3555,7 +3555,7 @@
       </c>
       <c r="K12" s="23"/>
       <c r="L12" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M12" s="23">
         <v>0</v>
@@ -3602,7 +3602,7 @@
         <v>79</v>
       </c>
       <c r="L13" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M13" s="23">
         <v>0</v>
@@ -3649,7 +3649,7 @@
         <v>84</v>
       </c>
       <c r="L14" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M14" s="23">
         <v>0</v>
@@ -3696,7 +3696,7 @@
         <v>87</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M15" s="23">
         <v>0</v>
@@ -3743,7 +3743,7 @@
         <v>90</v>
       </c>
       <c r="L16" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M16" s="23">
         <v>0</v>
@@ -3790,7 +3790,7 @@
         <v>93</v>
       </c>
       <c r="L17" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M17" s="23">
         <v>0</v>
@@ -3837,7 +3837,7 @@
         <v>96</v>
       </c>
       <c r="L18" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M18" s="23">
         <v>0</v>
@@ -3884,7 +3884,7 @@
         <v>99</v>
       </c>
       <c r="L19" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M19" s="23">
         <v>0</v>
@@ -3931,7 +3931,7 @@
         <v>102</v>
       </c>
       <c r="L20" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M20" s="23">
         <v>0</v>
@@ -3978,7 +3978,7 @@
         <v>105</v>
       </c>
       <c r="L21" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M21" s="23">
         <v>0</v>
@@ -4025,7 +4025,7 @@
         <v>108</v>
       </c>
       <c r="L22" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M22" s="23">
         <v>0</v>
@@ -4072,7 +4072,7 @@
         <v>111</v>
       </c>
       <c r="L23" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M23" s="23">
         <v>0</v>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="K24" s="23"/>
       <c r="L24" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M24" s="23">
         <v>0</v>
@@ -4164,7 +4164,7 @@
         <v>117</v>
       </c>
       <c r="L25" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M25" s="23">
         <v>0</v>
@@ -4211,7 +4211,7 @@
         <v>121</v>
       </c>
       <c r="L26" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M26" s="23">
         <v>0</v>
@@ -4258,7 +4258,7 @@
         <v>124</v>
       </c>
       <c r="L27" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M27" s="23">
         <v>0</v>
@@ -4305,7 +4305,7 @@
         <v>127</v>
       </c>
       <c r="L28" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M28" s="23">
         <v>0</v>
@@ -4352,7 +4352,7 @@
         <v>130</v>
       </c>
       <c r="L29" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M29" s="23">
         <v>0</v>
@@ -4399,7 +4399,7 @@
         <v>133</v>
       </c>
       <c r="L30" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M30" s="23">
         <v>0</v>
@@ -4446,7 +4446,7 @@
         <v>136</v>
       </c>
       <c r="L31" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M31" s="23">
         <v>0</v>
@@ -4493,7 +4493,7 @@
         <v>139</v>
       </c>
       <c r="L32" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M32" s="23">
         <v>0</v>
@@ -4540,7 +4540,7 @@
         <v>142</v>
       </c>
       <c r="L33" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M33" s="23">
         <v>0</v>
@@ -4587,7 +4587,7 @@
         <v>145</v>
       </c>
       <c r="L34" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M34" s="23">
         <v>0</v>
@@ -4634,7 +4634,7 @@
         <v>148</v>
       </c>
       <c r="L35" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M35" s="23">
         <v>0</v>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="K36" s="23"/>
       <c r="L36" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M36" s="23">
         <v>0</v>
@@ -4726,7 +4726,7 @@
         <v>154</v>
       </c>
       <c r="L37" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M37" s="23">
         <v>0</v>
@@ -4773,7 +4773,7 @@
         <v>159</v>
       </c>
       <c r="L38" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M38" s="23">
         <v>0</v>
@@ -4820,7 +4820,7 @@
         <v>162</v>
       </c>
       <c r="L39" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M39" s="23">
         <v>0</v>
@@ -4867,7 +4867,7 @@
         <v>165</v>
       </c>
       <c r="L40" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M40" s="23">
         <v>0</v>
@@ -4914,7 +4914,7 @@
         <v>168</v>
       </c>
       <c r="L41" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M41" s="23">
         <v>0</v>
@@ -4961,7 +4961,7 @@
         <v>171</v>
       </c>
       <c r="L42" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M42" s="23">
         <v>0</v>
@@ -5008,7 +5008,7 @@
         <v>174</v>
       </c>
       <c r="L43" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M43" s="23">
         <v>0</v>
@@ -5055,7 +5055,7 @@
         <v>177</v>
       </c>
       <c r="L44" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M44" s="23">
         <v>0</v>
@@ -5102,7 +5102,7 @@
         <v>180</v>
       </c>
       <c r="L45" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M45" s="23">
         <v>0</v>
@@ -5149,7 +5149,7 @@
         <v>183</v>
       </c>
       <c r="L46" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M46" s="23">
         <v>0</v>
@@ -5196,7 +5196,7 @@
         <v>186</v>
       </c>
       <c r="L47" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M47" s="23">
         <v>0</v>
@@ -5243,7 +5243,7 @@
         <v>189</v>
       </c>
       <c r="L48" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M48" s="23">
         <v>0</v>
@@ -5290,7 +5290,7 @@
         <v>192</v>
       </c>
       <c r="L49" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M49" s="23">
         <v>0</v>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="K50" s="23"/>
       <c r="L50" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M50" s="23">
         <v>0</v>
@@ -5382,7 +5382,7 @@
         <v>198</v>
       </c>
       <c r="L51" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M51" s="23">
         <v>0</v>
@@ -5429,7 +5429,7 @@
         <v>204</v>
       </c>
       <c r="L52" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M52" s="23">
         <v>0</v>
@@ -5476,7 +5476,7 @@
         <v>207</v>
       </c>
       <c r="L53" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M53" s="23">
         <v>0</v>
@@ -5523,7 +5523,7 @@
         <v>210</v>
       </c>
       <c r="L54" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M54" s="23">
         <v>0</v>
@@ -5570,7 +5570,7 @@
         <v>213</v>
       </c>
       <c r="L55" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M55" s="23">
         <v>0</v>
@@ -5617,7 +5617,7 @@
         <v>216</v>
       </c>
       <c r="L56" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M56" s="23">
         <v>0</v>
@@ -5664,7 +5664,7 @@
         <v>219</v>
       </c>
       <c r="L57" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M57" s="23">
         <v>0</v>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="K58" s="23"/>
       <c r="L58" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M58" s="23">
         <v>0</v>
@@ -5756,7 +5756,7 @@
         <v>225</v>
       </c>
       <c r="L59" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M59" s="23">
         <v>0</v>
@@ -5803,7 +5803,7 @@
         <v>229</v>
       </c>
       <c r="L60" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M60" s="23">
         <v>0</v>
@@ -5850,7 +5850,7 @@
         <v>232</v>
       </c>
       <c r="L61" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M61" s="23">
         <v>0</v>
@@ -5897,7 +5897,7 @@
         <v>235</v>
       </c>
       <c r="L62" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M62" s="23">
         <v>0</v>
@@ -5944,7 +5944,7 @@
         <v>238</v>
       </c>
       <c r="L63" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M63" s="23">
         <v>0</v>
@@ -5991,7 +5991,7 @@
         <v>241</v>
       </c>
       <c r="L64" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M64" s="23">
         <v>0</v>
@@ -6038,7 +6038,7 @@
         <v>244</v>
       </c>
       <c r="L65" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M65" s="23">
         <v>0</v>
@@ -6085,7 +6085,7 @@
         <v>247</v>
       </c>
       <c r="L66" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M66" s="23">
         <v>0</v>
@@ -6132,7 +6132,7 @@
         <v>250</v>
       </c>
       <c r="L67" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M67" s="23">
         <v>0</v>
@@ -6179,7 +6179,7 @@
         <v>253</v>
       </c>
       <c r="L68" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M68" s="23">
         <v>0</v>
@@ -6226,7 +6226,7 @@
         <v>256</v>
       </c>
       <c r="L69" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M69" s="23">
         <v>0</v>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="K70" s="23"/>
       <c r="L70" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M70" s="23">
         <v>0</v>
@@ -6318,7 +6318,7 @@
         <v>262</v>
       </c>
       <c r="L71" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M71" s="23">
         <v>0</v>
@@ -6365,7 +6365,7 @@
         <v>266</v>
       </c>
       <c r="L72" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M72" s="23">
         <v>0</v>
@@ -6412,7 +6412,7 @@
         <v>269</v>
       </c>
       <c r="L73" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M73" s="23">
         <v>0</v>
@@ -6459,7 +6459,7 @@
         <v>272</v>
       </c>
       <c r="L74" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M74" s="23">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>275</v>
       </c>
       <c r="L75" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M75" s="23">
         <v>0</v>
@@ -6553,7 +6553,7 @@
         <v>278</v>
       </c>
       <c r="L76" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M76" s="23">
         <v>0</v>
@@ -6600,7 +6600,7 @@
         <v>281</v>
       </c>
       <c r="L77" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M77" s="23">
         <v>0</v>
@@ -6647,7 +6647,7 @@
         <v>284</v>
       </c>
       <c r="L78" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M78" s="23">
         <v>0</v>
@@ -6692,7 +6692,7 @@
       </c>
       <c r="K79" s="23"/>
       <c r="L79" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M79" s="23">
         <v>0</v>
@@ -6739,7 +6739,7 @@
         <v>290</v>
       </c>
       <c r="L80" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M80" s="23">
         <v>0</v>
@@ -6786,7 +6786,7 @@
         <v>294</v>
       </c>
       <c r="L81" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M81" s="23">
         <v>0</v>
@@ -6833,7 +6833,7 @@
         <v>297</v>
       </c>
       <c r="L82" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M82" s="23">
         <v>0</v>
@@ -6880,7 +6880,7 @@
         <v>300</v>
       </c>
       <c r="L83" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M83" s="23">
         <v>0</v>
@@ -6927,7 +6927,7 @@
         <v>303</v>
       </c>
       <c r="L84" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M84" s="23">
         <v>0</v>
@@ -6974,7 +6974,7 @@
         <v>306</v>
       </c>
       <c r="L85" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M85" s="23">
         <v>0</v>
@@ -7021,7 +7021,7 @@
         <v>309</v>
       </c>
       <c r="L86" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M86" s="23">
         <v>0</v>
@@ -7068,7 +7068,7 @@
         <v>312</v>
       </c>
       <c r="L87" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M87" s="23">
         <v>0</v>
@@ -7115,7 +7115,7 @@
         <v>315</v>
       </c>
       <c r="L88" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M88" s="23">
         <v>0</v>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="K89" s="23"/>
       <c r="L89" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M89" s="23">
         <v>0</v>
@@ -7207,7 +7207,7 @@
         <v>321</v>
       </c>
       <c r="L90" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M90" s="23">
         <v>0</v>
@@ -7254,7 +7254,7 @@
         <v>325</v>
       </c>
       <c r="L91" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M91" s="23">
         <v>0</v>
@@ -7301,7 +7301,7 @@
         <v>328</v>
       </c>
       <c r="L92" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M92" s="23">
         <v>0</v>
@@ -7348,7 +7348,7 @@
         <v>331</v>
       </c>
       <c r="L93" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M93" s="23">
         <v>0</v>
@@ -7395,7 +7395,7 @@
         <v>334</v>
       </c>
       <c r="L94" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M94" s="23">
         <v>0</v>
@@ -7442,7 +7442,7 @@
         <v>337</v>
       </c>
       <c r="L95" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M95" s="23">
         <v>0</v>
@@ -7489,7 +7489,7 @@
         <v>340</v>
       </c>
       <c r="L96" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M96" s="23">
         <v>0</v>
@@ -7536,7 +7536,7 @@
         <v>343</v>
       </c>
       <c r="L97" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M97" s="23">
         <v>0</v>
@@ -7581,7 +7581,7 @@
       </c>
       <c r="K98" s="23"/>
       <c r="L98" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M98" s="23">
         <v>0</v>
@@ -7628,7 +7628,7 @@
         <v>349</v>
       </c>
       <c r="L99" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M99" s="23">
         <v>0</v>
@@ -7675,7 +7675,7 @@
         <v>353</v>
       </c>
       <c r="L100" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M100" s="23">
         <v>0</v>
@@ -7722,7 +7722,7 @@
         <v>356</v>
       </c>
       <c r="L101" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M101" s="23">
         <v>0</v>
@@ -7769,7 +7769,7 @@
         <v>359</v>
       </c>
       <c r="L102" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M102" s="23">
         <v>0</v>
@@ -7816,7 +7816,7 @@
         <v>362</v>
       </c>
       <c r="L103" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M103" s="23">
         <v>0</v>
@@ -7863,7 +7863,7 @@
         <v>365</v>
       </c>
       <c r="L104" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M104" s="23">
         <v>0</v>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="K105" s="23"/>
       <c r="L105" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M105" s="23">
         <v>0</v>
@@ -7955,7 +7955,7 @@
         <v>371</v>
       </c>
       <c r="L106" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M106" s="23">
         <v>0</v>
@@ -8002,7 +8002,7 @@
         <v>376</v>
       </c>
       <c r="L107" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M107" s="23">
         <v>0</v>
@@ -8049,7 +8049,7 @@
         <v>379</v>
       </c>
       <c r="L108" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M108" s="23">
         <v>0</v>
@@ -8096,7 +8096,7 @@
         <v>382</v>
       </c>
       <c r="L109" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M109" s="23">
         <v>0</v>
@@ -8143,7 +8143,7 @@
         <v>385</v>
       </c>
       <c r="L110" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M110" s="23">
         <v>0</v>
@@ -8190,7 +8190,7 @@
         <v>388</v>
       </c>
       <c r="L111" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M111" s="23">
         <v>0</v>
@@ -8237,7 +8237,7 @@
         <v>391</v>
       </c>
       <c r="L112" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M112" s="23">
         <v>0</v>
@@ -8284,7 +8284,7 @@
         <v>394</v>
       </c>
       <c r="L113" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M113" s="23">
         <v>0</v>
@@ -8331,7 +8331,7 @@
         <v>397</v>
       </c>
       <c r="L114" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M114" s="23">
         <v>0</v>
@@ -8376,7 +8376,7 @@
       </c>
       <c r="K115" s="23"/>
       <c r="L115" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M115" s="23">
         <v>0</v>
@@ -8423,7 +8423,7 @@
         <v>403</v>
       </c>
       <c r="L116" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M116" s="23">
         <v>0</v>
@@ -8470,7 +8470,7 @@
         <v>408</v>
       </c>
       <c r="L117" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M117" s="23">
         <v>0</v>
@@ -8517,7 +8517,7 @@
         <v>411</v>
       </c>
       <c r="L118" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M118" s="23">
         <v>0</v>
@@ -8564,7 +8564,7 @@
         <v>414</v>
       </c>
       <c r="L119" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M119" s="23">
         <v>0</v>
@@ -8611,7 +8611,7 @@
         <v>417</v>
       </c>
       <c r="L120" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M120" s="23">
         <v>0</v>
@@ -8658,7 +8658,7 @@
         <v>420</v>
       </c>
       <c r="L121" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M121" s="23">
         <v>0</v>
@@ -8705,7 +8705,7 @@
         <v>423</v>
       </c>
       <c r="L122" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M122" s="23">
         <v>0</v>
@@ -8752,7 +8752,7 @@
         <v>426</v>
       </c>
       <c r="L123" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M123" s="23">
         <v>0</v>
@@ -8799,7 +8799,7 @@
         <v>429</v>
       </c>
       <c r="L124" s="23" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M124" s="23">
         <v>0</v>
@@ -8823,7 +8823,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" aboveAverage="0" operator="containsText" rank="0" text="Completed" id="{0D6ACE5B-3544-465C-B7CE-6B91FAE6D1CA}">
+          <x14:cfRule type="containsText" priority="2" aboveAverage="0" operator="containsText" rank="0" text="Completed" id="{9900F14E-E88E-4678-B37F-D2B18A80BDCB}">
             <xm:f>NOT(ISERROR(SEARCH("Completed",L2)))</xm:f>
             <x14:dxf>
               <font>
@@ -8841,7 +8841,7 @@
           <xm:sqref>L2:L124</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" aboveAverage="0" operator="containsText" rank="0" text="In Progress" id="{E5A2633F-FE6D-4336-8F75-DF11F90DC9F4}">
+          <x14:cfRule type="containsText" priority="3" aboveAverage="0" operator="containsText" rank="0" text="In Progress" id="{328A7771-2D67-4AF9-927B-F5168AEDC497}">
             <xm:f>NOT(ISERROR(SEARCH("In Progress",L2)))</xm:f>
             <x14:dxf>
               <font>
@@ -8858,7 +8858,7 @@
           <xm:sqref>L2:L124</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" aboveAverage="0" operator="containsText" rank="0" text="Revisit" id="{BA4E5BAD-3963-45B8-9C04-D3BD81E29477}">
+          <x14:cfRule type="containsText" priority="4" aboveAverage="0" operator="containsText" rank="0" text="Revisit" id="{D95E3601-8BBD-4AC2-8690-F9252B36512B}">
             <xm:f>NOT(ISERROR(SEARCH("Revisit",L2)))</xm:f>
             <x14:dxf>
               <font>
@@ -8875,7 +8875,7 @@
           <xm:sqref>L2:L124</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" priority="5" id="{D1B9B614-D747-4940-A57B-ECD921C404F4}">
+          <x14:cfRule type="dataBar" priority="5" id="{6FE29B43-BA9E-4E25-B324-55E9B9B9FD66}">
             <x14:dataBar maxLength="90" minLength="10" axisPosition="automatic" direction="context">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -8890,7 +8890,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{420FDE69-CEC2-44A1-AC4F-E2D53512F67D}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{776AAC6B-FEEC-4395-82D3-88E03D01DF9B}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"☐ Not Started,◐ In Progress,☑ Completed,↻ Revisit"</xm:f>
           </x14:formula1>
@@ -8899,7 +8899,7 @@
           </x14:formula2>
           <xm:sqref>L2:L124</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{96B9E689-C74A-45FE-96CE-2D9FC222556C}" type="whole" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{60F40BE6-F493-4A59-A361-5A88D59FABA0}" type="whole" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
@@ -9545,7 +9545,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{7C177C08-5769-42A1-8B49-358F5827E7E3}" type="decimal" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{A308CF30-536E-4B1F-BF91-43B0354036A4}" type="decimal" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
@@ -11016,7 +11016,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{D2A246AA-4F16-4E26-9D2B-D6FE2163F839}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{F5A6C0CF-EF64-4011-B35E-E0B3B77D0133}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Build,Troubleshoot,Rebuild,Timed Mock,Review"</xm:f>
           </x14:formula1>
@@ -11025,7 +11025,7 @@
           </x14:formula2>
           <xm:sqref>D2:D201</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{382C417B-8BC6-444A-BFEE-589C864C44C7}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{621BD406-F3F6-4FCF-BECB-8C0F543E05DD}" type="list" allowBlank="0" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Pass,Partial,Fail"</xm:f>
           </x14:formula1>
@@ -11304,7 +11304,7 @@
     </row>
     <row r="2" ht="15">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>

</xml_diff>